<commit_message>
fix(cierre): publicar planfrizze.xlsx + 2 clientes nuevos del Plan Frizze
El negocio agrego 1462 y 1463 a "Clientes activos" del xlsx y no aparecian
en el portal: el archivo nunca viajaba a Render. 01_INPUTS/PLAN FRIZZE no
estaba en el allowlist del cierre, y check_git_cierre.py lo da por bueno
porque cuelga de 01_INPUTS/, asi que el cierre cerraba en verde con el
cambio sin publicar (mismo patron que ERR-014 con dadatinto).

- CIERRE_DIA_ORBIT.bat: git add "01_INPUTS/PLAN FRIZZE/planfrizze.xlsx".
- Se publica el xlsx actual: 301, 1443, 1462, 1463.

Verificado en local: gerencia devuelve las 4 tarjetas; por vendedor,
V8 = 301 + 1462 + 1463 y V10 = 1443.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/PLAN FRIZZE/planfrizze.xlsx
+++ b/01_INPUTS/PLAN FRIZZE/planfrizze.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\PLAN FRIZZE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFD08DC0-06E2-448C-93AB-9332AEAB448B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374DE14-C394-4B5E-B881-CC57081DB977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{D0100D6D-D9A5-4948-99A8-36A5A8B33663}"/>
   </bookViews>
@@ -42,9 +42,6 @@
     <t>Acción: 3+1 en frizze de la misma variedad</t>
   </si>
   <si>
-    <t>Clientes activos: 301, 1443</t>
-  </si>
-  <si>
     <t>códigos productos que entran:(14583) FRIZZE BLUE NEW, (14619) FRIZZE BUBBLE MOOD</t>
   </si>
   <si>
@@ -52,6 +49,9 @@
   </si>
   <si>
     <t>Tope: 3 combos del Blue (osea: 9+3) y 3 combos del Bubble (osea 9+3) pack de 6 botellas</t>
+  </si>
+  <si>
+    <t>Clientes activos: 301, 1443, 1462, 1463</t>
   </si>
 </sst>
 </file>
@@ -421,22 +421,22 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>